<commit_message>
Add custom holidays, regressors, and XGBoost comparison
</commit_message>
<xml_diff>
--- a/sales_2024.xlsx
+++ b/sales_2024.xlsx
@@ -3,18 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30019"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="190" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2FDFD5E-302C-4B25-8C5D-CCF0A050E87E}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{391FB8E1-B9D5-411F-A898-7D2AA7969566}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="6" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jan 2024" sheetId="12" r:id="rId1"/>
     <sheet name="Feb 2024" sheetId="11" r:id="rId2"/>
-    <sheet name="March 2024" sheetId="10" r:id="rId3"/>
-    <sheet name="April 2024" sheetId="9" r:id="rId4"/>
+    <sheet name="Mar 2024" sheetId="10" r:id="rId3"/>
+    <sheet name="Apr 2024" sheetId="9" r:id="rId4"/>
     <sheet name="May 2024" sheetId="8" r:id="rId5"/>
-    <sheet name="June 2024" sheetId="7" r:id="rId6"/>
-    <sheet name="July 2024" sheetId="6" r:id="rId7"/>
+    <sheet name="Jun 2024" sheetId="7" r:id="rId6"/>
+    <sheet name="Jul 2024" sheetId="6" r:id="rId7"/>
     <sheet name="Aug 2024" sheetId="5" r:id="rId8"/>
     <sheet name="Sep 2024" sheetId="4" r:id="rId9"/>
     <sheet name="Oct 2024" sheetId="3" r:id="rId10"/>
@@ -1181,7 +1181,7 @@
         <v>45624</v>
       </c>
       <c r="B29" s="2">
-        <v>135.97999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">

</xml_diff>